<commit_message>
add column for acceptance criteria
</commit_message>
<xml_diff>
--- a/actual excel template/Test_Case_Template.xlsx
+++ b/actual excel template/Test_Case_Template.xlsx
@@ -1,129 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29803"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MarkJohnAjero\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F0740E8D-3A41-4F93-965D-F186E842C079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D48A89E6-1122-4D92-9EBD-16E60DBDD4A5}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Page1" sheetId="1" r:id="rId1"/>
+    <sheet name="Page1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
-  <si>
-    <t>TestCase ID</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Precondition</t>
-  </si>
-  <si>
-    <t>Steps to Reproduce</t>
-  </si>
-  <si>
-    <t>Expected Results</t>
-  </si>
-  <si>
-    <t>Actual Result</t>
-  </si>
-  <si>
-    <t>Status (Pass/Fail)</t>
-  </si>
-  <si>
-    <t>QA Tester</t>
-  </si>
-  <si>
-    <t>QA Notes</t>
-  </si>
-  <si>
-    <t>20262SP1-0001</t>
-  </si>
-  <si>
-    <t>Critical</t>
-  </si>
-  <si>
-    <t>Verify display of Events in Detection module</t>
-  </si>
-  <si>
-    <t>Environment must have a Malware or Malicious Activity</t>
-  </si>
-  <si>
-    <t>1. Log in to the EDR Aquila module.
-2. Navigate to the Cyber Monitoring &gt; Endpoint Detection and Response (EDR) &gt;  Detection.
-4. Select Events tab.
-3. Review Event list.</t>
-  </si>
-  <si>
-    <t>Detection alerts are displayed with correct severity, timestamp, and endpoint details.</t>
-  </si>
-  <si>
-    <t>Fail</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.89999084444715716"/>
+        <fgColor theme="3" tint="0.8999908444471572"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -141,12 +52,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -199,28 +110,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FFFF4F4F"/>
-      <color rgb="FF77C38B"/>
-      <color rgb="FFFF3300"/>
-      <color rgb="FFF4CE2C"/>
-      <color rgb="FFF9992F"/>
-      <color rgb="FFFC6E56"/>
-      <color rgb="FFFF7575"/>
-      <color rgb="FFFF8B8B"/>
-      <color rgb="FFFFA86D"/>
-      <color rgb="FFFF9797"/>
-    </mruColors>
-  </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors/>
 </styleSheet>
 </file>
 
@@ -540,149 +430,204 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5186A37D-C595-45B5-BD90-42BCF7B42D1D}">
-  <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="73" customWidth="1"/>
-    <col min="4" max="6" width="45.5703125" customWidth="1"/>
-    <col min="7" max="7" width="45.42578125" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" customWidth="1"/>
-    <col min="9" max="9" width="36.7109375" customWidth="1"/>
-    <col min="10" max="10" width="36.85546875" customWidth="1"/>
+    <col width="18.28515625" customWidth="1" min="1" max="2"/>
+    <col width="73" customWidth="1" min="3" max="3"/>
+    <col width="45.5703125" customWidth="1" min="4" max="6"/>
+    <col width="45.42578125" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
+    <row r="1" customFormat="1" s="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>TestCase ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Steps to Reproduce</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Status (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>QA Tester</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>QA Notes</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="75">
-      <c r="A2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+    <row r="2" ht="75" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>20262SP1-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Verify display of Events in Detection module</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Environment must have a Malware or Malicious Activity</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in to the EDR Aquila module.
+2. Navigate to the Cyber Monitoring &gt; Endpoint Detection and Response (EDR) &gt;  Detection.
+4. Select Events tab.
+3. Review Event list.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Detection alerts are displayed with correct severity, timestamp, and endpoint details.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
     </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+    <row r="4">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
     </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1:B6 B8:B1048576">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Low"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="6" operator="equal">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:H1048576">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1:H1048576" xr:uid="{17C587A8-1A48-44A0-A450-A3F91A90C00D}">
+    <dataValidation sqref="H1:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:B1048576 B1:B6" xr:uid="{EED69826-97FC-4224-B1BB-9FCCA6EFBB84}">
+    <dataValidation sqref="B1:B6 B8:B1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Critical, High, Medium, Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>